<commit_message>
Update bug collection commit log
</commit_message>
<xml_diff>
--- a/commits-log.xlsx
+++ b/commits-log.xlsx
@@ -13,11 +13,11 @@
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="38" customWidth="1"/>
+    <col min="4" max="4" width="42" customWidth="1"/>
     <col min="5" max="5" width="46" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="34" customWidth="1"/>
-    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="6" max="6" width="44" customWidth="1"/>
+    <col min="7" max="7" width="30" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -70,7 +70,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>待补</t>
+          <t>#6</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -90,17 +90,17 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>src/main.cpp</t>
+          <t>src/main.cpp; bug-collection/issue-001/README.md</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>568865a 或实际 PR 合入 commit</t>
+          <t>dc70bd9 / merge 428de6d</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>待创建 Issue/PR</t>
+          <t>已合入 main</t>
         </is>
       </c>
     </row>
@@ -112,7 +112,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>待补</t>
+          <t>#7</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -132,17 +132,17 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>src/main.cpp</t>
+          <t>src/main.cpp; bug-collection/issue-002/README.md</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>248743d 或实际 PR 合入 commit</t>
+          <t>db97fd4 / merge b7ebc39</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>待创建 Issue/PR</t>
+          <t>已合入 main</t>
         </is>
       </c>
     </row>
@@ -154,7 +154,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>待补</t>
+          <t>#8</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>src/main.cpp</t>
+          <t>src/main.cpp; bug-collection/issue-003/README.md</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>568865a 或实际 PR 合入 commit</t>
+          <t>40a1fae / merge 68efd93</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>待创建 Issue/PR</t>
+          <t>已合入 main</t>
         </is>
       </c>
     </row>
@@ -196,7 +196,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>待补</t>
+          <t>#9</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -216,17 +216,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>src/main.cpp</t>
+          <t>src/main.cpp; bug-collection/issue-004/README.md</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>634b1d7 或实际 PR 合入 commit</t>
+          <t>bf3975e / merge 45678cc</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>待创建 Issue/PR</t>
+          <t>已合入 main</t>
         </is>
       </c>
     </row>
@@ -238,7 +238,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>待补</t>
+          <t>#10</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -258,17 +258,17 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>src/main.cpp</t>
+          <t>src/main.cpp; bug-collection/issue-005/README.md</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>634b1d7 或实际 PR 合入 commit</t>
+          <t>2399f1b / merge 98afee8</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>待创建 Issue/PR</t>
+          <t>已合入 main</t>
         </is>
       </c>
     </row>

</xml_diff>